<commit_message>
laga aðeins í measurements excelinu og svo bæta inn mynd, video og description fyrir t-test til að testa
</commit_message>
<xml_diff>
--- a/measurementInfo.xlsx
+++ b/measurementInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Notandi\Desktop\Measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89EABDE-47D2-4DB6-8407-B51989CF139A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{113F60A8-B43A-4B24-92E7-501643F71727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5685" windowWidth="16440" windowHeight="28320" xr2:uid="{CE7ABF46-5BCF-44D0-B551-448571CF2DF6}"/>
+    <workbookView xWindow="7095" yWindow="2340" windowWidth="16410" windowHeight="11295" xr2:uid="{CE7ABF46-5BCF-44D0-B551-448571CF2DF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -401,12 +401,6 @@
     <t>soccer_penalty_box_wide_dribbling</t>
   </si>
   <si>
-    <t>soccer_shooting_douple_shooting</t>
-  </si>
-  <si>
-    <t>soccer_shooting_triple_shoooting</t>
-  </si>
-  <si>
     <t>soccer_sprint_one_gate_generic</t>
   </si>
   <si>
@@ -623,9 +617,6 @@
     <t>soccer_yoyo_interm_recover_test_level_2</t>
   </si>
   <si>
-    <t>soccer_five_times_30m_generic</t>
-  </si>
-  <si>
     <t>soccer_five_time_30m_sprint</t>
   </si>
   <si>
@@ -645,6 +636,15 @@
   </si>
   <si>
     <t>Key</t>
+  </si>
+  <si>
+    <t>soccer_shooting_triple_shooting</t>
+  </si>
+  <si>
+    <t>soccer_shooting_double_shooting</t>
+  </si>
+  <si>
+    <t>soccer_five_time_30m_generic</t>
   </si>
 </sst>
 </file>
@@ -1077,10 +1077,10 @@
         <v>77</v>
       </c>
       <c r="H2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1106,10 +1106,10 @@
         <v>77</v>
       </c>
       <c r="H3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1135,10 +1135,10 @@
         <v>77</v>
       </c>
       <c r="H4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -1164,10 +1164,10 @@
         <v>77</v>
       </c>
       <c r="H5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I5" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1187,10 +1187,10 @@
         <v>77</v>
       </c>
       <c r="H6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I6" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1213,13 +1213,13 @@
         <v>91</v>
       </c>
       <c r="G7" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="H7" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I7" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1245,10 +1245,10 @@
         <v>93</v>
       </c>
       <c r="H8" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="I8" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1274,10 +1274,10 @@
         <v>93</v>
       </c>
       <c r="H9" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I9" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -1303,10 +1303,10 @@
         <v>98</v>
       </c>
       <c r="H10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I10" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -1332,10 +1332,10 @@
         <v>98</v>
       </c>
       <c r="H11" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I11" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -1361,10 +1361,10 @@
         <v>98</v>
       </c>
       <c r="H12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I12" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -1390,10 +1390,10 @@
         <v>77</v>
       </c>
       <c r="H13" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -1419,10 +1419,10 @@
         <v>77</v>
       </c>
       <c r="H14" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I14" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1448,10 +1448,10 @@
         <v>93</v>
       </c>
       <c r="H15" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="I15" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1477,10 +1477,10 @@
         <v>93</v>
       </c>
       <c r="H16" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="I16" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -1506,10 +1506,10 @@
         <v>98</v>
       </c>
       <c r="H17" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I17" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -1535,10 +1535,10 @@
         <v>98</v>
       </c>
       <c r="H18" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="I18" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -1564,10 +1564,10 @@
         <v>98</v>
       </c>
       <c r="H19" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I19" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -1593,10 +1593,10 @@
         <v>98</v>
       </c>
       <c r="H20" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="I20" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -1622,10 +1622,10 @@
         <v>98</v>
       </c>
       <c r="H21" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I21" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -1651,10 +1651,10 @@
         <v>98</v>
       </c>
       <c r="H22" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I22" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -1680,10 +1680,10 @@
         <v>98</v>
       </c>
       <c r="H23" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="I23" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -1709,10 +1709,10 @@
         <v>98</v>
       </c>
       <c r="H24" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="I24" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -1723,7 +1723,7 @@
         <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>121</v>
+        <v>201</v>
       </c>
       <c r="D25" t="s">
         <v>82</v>
@@ -1738,10 +1738,10 @@
         <v>98</v>
       </c>
       <c r="H25" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I25" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -1752,7 +1752,7 @@
         <v>33</v>
       </c>
       <c r="C26" t="s">
-        <v>122</v>
+        <v>200</v>
       </c>
       <c r="D26" t="s">
         <v>82</v>
@@ -1767,10 +1767,10 @@
         <v>98</v>
       </c>
       <c r="H26" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I26" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -1778,7 +1778,7 @@
         <v>34</v>
       </c>
       <c r="C27" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -1789,7 +1789,7 @@
         <v>35</v>
       </c>
       <c r="C28" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D28" t="s">
         <v>77</v>
@@ -1801,13 +1801,13 @@
         <v>91</v>
       </c>
       <c r="G28" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="H28" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="I28" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -1818,7 +1818,7 @@
         <v>36</v>
       </c>
       <c r="C29" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D29" t="s">
         <v>82</v>
@@ -1833,10 +1833,10 @@
         <v>98</v>
       </c>
       <c r="H29" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I29" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -1844,10 +1844,10 @@
         <v>37</v>
       </c>
       <c r="B30" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C30" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D30" t="s">
         <v>77</v>
@@ -1862,10 +1862,10 @@
         <v>93</v>
       </c>
       <c r="H30" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I30" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -1873,10 +1873,10 @@
         <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C31" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D31" t="s">
         <v>82</v>
@@ -1891,10 +1891,10 @@
         <v>98</v>
       </c>
       <c r="H31" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I31" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -1902,10 +1902,10 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C32" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D32" t="s">
         <v>77</v>
@@ -1920,10 +1920,10 @@
         <v>98</v>
       </c>
       <c r="H32" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I32" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -1934,7 +1934,7 @@
         <v>40</v>
       </c>
       <c r="C33" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D33" t="s">
         <v>82</v>
@@ -1946,13 +1946,13 @@
         <v>88</v>
       </c>
       <c r="G33" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="H33" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="I33" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -1963,22 +1963,22 @@
         <v>41</v>
       </c>
       <c r="C34" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D34" t="s">
         <v>77</v>
       </c>
       <c r="E34" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G34" t="s">
         <v>77</v>
       </c>
       <c r="H34" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I34" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -1986,7 +1986,7 @@
         <v>42</v>
       </c>
       <c r="C35" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -1994,10 +1994,10 @@
         <v>43</v>
       </c>
       <c r="B36" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C36" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D36" t="s">
         <v>82</v>
@@ -2012,10 +2012,10 @@
         <v>93</v>
       </c>
       <c r="H36" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I36" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -2023,10 +2023,10 @@
         <v>44</v>
       </c>
       <c r="B37" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D37" t="s">
         <v>77</v>
@@ -2041,10 +2041,10 @@
         <v>93</v>
       </c>
       <c r="H37" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I37" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -2052,10 +2052,10 @@
         <v>45</v>
       </c>
       <c r="B38" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C38" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D38" t="s">
         <v>82</v>
@@ -2070,10 +2070,10 @@
         <v>98</v>
       </c>
       <c r="H38" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I38" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -2081,10 +2081,10 @@
         <v>46</v>
       </c>
       <c r="B39" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C39" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D39" t="s">
         <v>77</v>
@@ -2099,10 +2099,10 @@
         <v>98</v>
       </c>
       <c r="H39" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I39" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -2110,10 +2110,10 @@
         <v>47</v>
       </c>
       <c r="B40" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C40" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D40" t="s">
         <v>82</v>
@@ -2128,10 +2128,10 @@
         <v>98</v>
       </c>
       <c r="H40" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I40" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -2139,10 +2139,10 @@
         <v>48</v>
       </c>
       <c r="B41" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C41" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D41" t="s">
         <v>77</v>
@@ -2157,10 +2157,10 @@
         <v>98</v>
       </c>
       <c r="H41" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I41" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -2168,10 +2168,10 @@
         <v>49</v>
       </c>
       <c r="B42" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C42" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D42" t="s">
         <v>82</v>
@@ -2186,10 +2186,10 @@
         <v>98</v>
       </c>
       <c r="H42" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I42" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -2197,10 +2197,10 @@
         <v>50</v>
       </c>
       <c r="B43" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C43" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D43" t="s">
         <v>77</v>
@@ -2215,10 +2215,10 @@
         <v>98</v>
       </c>
       <c r="H43" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I43" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -2226,10 +2226,10 @@
         <v>51</v>
       </c>
       <c r="B44" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C44" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D44" t="s">
         <v>82</v>
@@ -2244,10 +2244,10 @@
         <v>93</v>
       </c>
       <c r="H44" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I44" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -2255,10 +2255,10 @@
         <v>52</v>
       </c>
       <c r="B45" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D45" t="s">
         <v>77</v>
@@ -2270,13 +2270,13 @@
         <v>79</v>
       </c>
       <c r="G45" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="H45" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I45" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -2284,22 +2284,22 @@
         <v>53</v>
       </c>
       <c r="C46" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D46" t="s">
         <v>77</v>
       </c>
       <c r="E46" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G46" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H46" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I46" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -2307,10 +2307,10 @@
         <v>54</v>
       </c>
       <c r="B47" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C47" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D47" t="s">
         <v>82</v>
@@ -2325,10 +2325,10 @@
         <v>98</v>
       </c>
       <c r="H47" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I47" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -2336,10 +2336,10 @@
         <v>55</v>
       </c>
       <c r="B48" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C48" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D48" t="s">
         <v>77</v>
@@ -2354,10 +2354,10 @@
         <v>98</v>
       </c>
       <c r="H48" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I48" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
@@ -2365,10 +2365,10 @@
         <v>56</v>
       </c>
       <c r="B49" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C49" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D49" t="s">
         <v>82</v>
@@ -2383,10 +2383,10 @@
         <v>98</v>
       </c>
       <c r="H49" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I49" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -2394,10 +2394,10 @@
         <v>57</v>
       </c>
       <c r="B50" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C50" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D50" t="s">
         <v>77</v>
@@ -2412,10 +2412,10 @@
         <v>93</v>
       </c>
       <c r="H50" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I50" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -2423,10 +2423,10 @@
         <v>58</v>
       </c>
       <c r="B51" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C51" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D51" t="s">
         <v>82</v>
@@ -2441,10 +2441,10 @@
         <v>98</v>
       </c>
       <c r="H51" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I51" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -2452,10 +2452,10 @@
         <v>59</v>
       </c>
       <c r="B52" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C52" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D52" t="s">
         <v>77</v>
@@ -2470,10 +2470,10 @@
         <v>98</v>
       </c>
       <c r="H52" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I52" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -2484,7 +2484,7 @@
         <v>60</v>
       </c>
       <c r="C53" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D53" t="s">
         <v>77</v>
@@ -2499,10 +2499,10 @@
         <v>98</v>
       </c>
       <c r="H53" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I53" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -2510,7 +2510,7 @@
         <v>61</v>
       </c>
       <c r="C54" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -2518,10 +2518,10 @@
         <v>62</v>
       </c>
       <c r="B55" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C55" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D55" t="s">
         <v>77</v>
@@ -2536,10 +2536,10 @@
         <v>98</v>
       </c>
       <c r="H55" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I55" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -2547,10 +2547,10 @@
         <v>63</v>
       </c>
       <c r="B56" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C56" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D56" t="s">
         <v>82</v>
@@ -2570,10 +2570,10 @@
         <v>64</v>
       </c>
       <c r="B57" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C57" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D57" t="s">
         <v>77</v>
@@ -2588,10 +2588,10 @@
         <v>98</v>
       </c>
       <c r="H57" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I57" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -2599,7 +2599,7 @@
         <v>65</v>
       </c>
       <c r="C58" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -2607,16 +2607,16 @@
         <v>66</v>
       </c>
       <c r="B59" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C59" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D59" t="s">
         <v>77</v>
       </c>
       <c r="E59" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F59" t="s">
         <v>79</v>
@@ -2625,10 +2625,10 @@
         <v>77</v>
       </c>
       <c r="H59" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I59" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -2636,7 +2636,7 @@
         <v>67</v>
       </c>
       <c r="C60" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -2644,10 +2644,10 @@
         <v>68</v>
       </c>
       <c r="B61" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C61" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D61" t="s">
         <v>77</v>
@@ -2662,10 +2662,10 @@
         <v>98</v>
       </c>
       <c r="H61" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I61" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -2673,10 +2673,10 @@
         <v>69</v>
       </c>
       <c r="B62" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C62" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D62" t="s">
         <v>77</v>
@@ -2691,10 +2691,10 @@
         <v>98</v>
       </c>
       <c r="H62" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I62" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -2702,10 +2702,10 @@
         <v>70</v>
       </c>
       <c r="B63" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C63" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D63" t="s">
         <v>77</v>
@@ -2720,10 +2720,10 @@
         <v>98</v>
       </c>
       <c r="H63" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I63" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -2731,10 +2731,10 @@
         <v>71</v>
       </c>
       <c r="B64" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C64" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D64" t="s">
         <v>77</v>
@@ -2749,10 +2749,10 @@
         <v>98</v>
       </c>
       <c r="H64" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I64" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -2760,10 +2760,10 @@
         <v>72</v>
       </c>
       <c r="B65" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C65" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D65" t="s">
         <v>77</v>
@@ -2778,10 +2778,10 @@
         <v>93</v>
       </c>
       <c r="H65" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I65" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -2789,10 +2789,10 @@
         <v>73</v>
       </c>
       <c r="B66" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C66" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D66" t="s">
         <v>77</v>
@@ -2807,10 +2807,10 @@
         <v>98</v>
       </c>
       <c r="H66" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I66" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -2818,7 +2818,7 @@
         <v>74</v>
       </c>
       <c r="C67" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
@@ -2826,22 +2826,22 @@
         <v>74</v>
       </c>
       <c r="C68" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="E68" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F68" t="s">
         <v>79</v>
       </c>
       <c r="G68" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="H68" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I68" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
gera imagelrg fyrir allt
</commit_message>
<xml_diff>
--- a/measurementInfo.xlsx
+++ b/measurementInfo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Notandi\Desktop\Measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AABE33D-7259-4781-8E8B-67D77D864DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA60187-614B-4CBC-AB5C-D746FE7D08B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CE7ABF46-5BCF-44D0-B551-448571CF2DF6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="192">
   <si>
     <t>title</t>
   </si>
@@ -570,9 +570,6 @@
   </si>
   <si>
     <t>soccer_five_time_30m_sprint</t>
-  </si>
-  <si>
-    <t>Not available</t>
   </si>
   <si>
     <t>Premium</t>
@@ -1050,7 +1047,7 @@
         <v>125</v>
       </c>
       <c r="I2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1079,15 +1076,15 @@
         <v>125</v>
       </c>
       <c r="I3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" t="s">
         <v>186</v>
-      </c>
-      <c r="B4" t="s">
-        <v>187</v>
       </c>
       <c r="C4" t="s">
         <v>79</v>
@@ -1108,7 +1105,7 @@
         <v>125</v>
       </c>
       <c r="I4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -1137,7 +1134,7 @@
         <v>125</v>
       </c>
       <c r="I5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1160,7 +1157,7 @@
         <v>125</v>
       </c>
       <c r="I6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1183,13 +1180,13 @@
         <v>85</v>
       </c>
       <c r="G7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1215,10 +1212,10 @@
         <v>87</v>
       </c>
       <c r="H8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1244,10 +1241,10 @@
         <v>87</v>
       </c>
       <c r="H9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -1276,7 +1273,7 @@
         <v>125</v>
       </c>
       <c r="I10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -1302,10 +1299,10 @@
         <v>92</v>
       </c>
       <c r="H11" t="s">
+        <v>178</v>
+      </c>
+      <c r="I11" t="s">
         <v>179</v>
-      </c>
-      <c r="I11" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -1334,7 +1331,7 @@
         <v>125</v>
       </c>
       <c r="I12" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -1363,7 +1360,7 @@
         <v>125</v>
       </c>
       <c r="I13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -1392,7 +1389,7 @@
         <v>125</v>
       </c>
       <c r="I14" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -1418,10 +1415,10 @@
         <v>87</v>
       </c>
       <c r="H15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1447,10 +1444,10 @@
         <v>87</v>
       </c>
       <c r="H16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -1461,7 +1458,7 @@
         <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D17" t="s">
         <v>77</v>
@@ -1476,10 +1473,10 @@
         <v>92</v>
       </c>
       <c r="H17" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I17" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -1505,10 +1502,10 @@
         <v>92</v>
       </c>
       <c r="H18" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I18" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -1534,10 +1531,10 @@
         <v>92</v>
       </c>
       <c r="H19" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I19" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -1563,10 +1560,10 @@
         <v>92</v>
       </c>
       <c r="H20" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I20" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -1592,10 +1589,10 @@
         <v>92</v>
       </c>
       <c r="H21" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I21" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -1621,10 +1618,10 @@
         <v>92</v>
       </c>
       <c r="H22" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I22" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -1650,10 +1647,10 @@
         <v>92</v>
       </c>
       <c r="H23" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I23" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -1679,10 +1676,10 @@
         <v>92</v>
       </c>
       <c r="H24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -1693,7 +1690,7 @@
         <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D25" t="s">
         <v>77</v>
@@ -1708,10 +1705,10 @@
         <v>92</v>
       </c>
       <c r="H25" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I25" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -1722,7 +1719,7 @@
         <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D26" t="s">
         <v>77</v>
@@ -1737,10 +1734,10 @@
         <v>92</v>
       </c>
       <c r="H26" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I26" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -1763,13 +1760,13 @@
         <v>85</v>
       </c>
       <c r="G27" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H27" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I27" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -1798,7 +1795,7 @@
         <v>125</v>
       </c>
       <c r="I28" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -1824,10 +1821,10 @@
         <v>87</v>
       </c>
       <c r="H29" t="s">
+        <v>178</v>
+      </c>
+      <c r="I29" t="s">
         <v>179</v>
-      </c>
-      <c r="I29" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -1856,7 +1853,7 @@
         <v>125</v>
       </c>
       <c r="I30" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -1885,7 +1882,7 @@
         <v>125</v>
       </c>
       <c r="I31" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -1908,13 +1905,13 @@
         <v>82</v>
       </c>
       <c r="G32" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H32" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I32" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -1966,10 +1963,10 @@
         <v>87</v>
       </c>
       <c r="H34" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I34" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -1995,10 +1992,10 @@
         <v>87</v>
       </c>
       <c r="H35" t="s">
+        <v>178</v>
+      </c>
+      <c r="I35" t="s">
         <v>179</v>
-      </c>
-      <c r="I35" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -2027,7 +2024,7 @@
         <v>125</v>
       </c>
       <c r="I36" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -2056,7 +2053,7 @@
         <v>125</v>
       </c>
       <c r="I37" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -2082,10 +2079,10 @@
         <v>92</v>
       </c>
       <c r="H38" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I38" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -2114,7 +2111,7 @@
         <v>125</v>
       </c>
       <c r="I39" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -2143,7 +2140,7 @@
         <v>125</v>
       </c>
       <c r="I40" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -2172,7 +2169,7 @@
         <v>125</v>
       </c>
       <c r="I41" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -2201,7 +2198,7 @@
         <v>125</v>
       </c>
       <c r="I42" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -2224,13 +2221,13 @@
         <v>74</v>
       </c>
       <c r="G43" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H43" t="s">
         <v>125</v>
       </c>
       <c r="I43" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -2247,13 +2244,13 @@
         <v>147</v>
       </c>
       <c r="G44" t="s">
-        <v>147</v>
+        <v>72</v>
       </c>
       <c r="H44" t="s">
         <v>125</v>
       </c>
       <c r="I44" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -2282,7 +2279,7 @@
         <v>125</v>
       </c>
       <c r="I45" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -2311,7 +2308,7 @@
         <v>125</v>
       </c>
       <c r="I46" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -2340,7 +2337,7 @@
         <v>125</v>
       </c>
       <c r="I47" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -2369,7 +2366,7 @@
         <v>125</v>
       </c>
       <c r="I48" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
@@ -2398,7 +2395,7 @@
         <v>125</v>
       </c>
       <c r="I49" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -2427,7 +2424,7 @@
         <v>125</v>
       </c>
       <c r="I50" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -2456,7 +2453,7 @@
         <v>125</v>
       </c>
       <c r="I51" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
@@ -2485,7 +2482,7 @@
         <v>125</v>
       </c>
       <c r="I52" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -2537,7 +2534,7 @@
         <v>125</v>
       </c>
       <c r="I54" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -2566,7 +2563,7 @@
         <v>125</v>
       </c>
       <c r="I55" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -2595,7 +2592,7 @@
         <v>125</v>
       </c>
       <c r="I56" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -2624,7 +2621,7 @@
         <v>125</v>
       </c>
       <c r="I57" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -2635,7 +2632,7 @@
         <v>173</v>
       </c>
       <c r="C58" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D58" t="s">
         <v>72</v>
@@ -2653,7 +2650,7 @@
         <v>125</v>
       </c>
       <c r="I58" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -2664,7 +2661,7 @@
         <v>174</v>
       </c>
       <c r="C59" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D59" t="s">
         <v>72</v>
@@ -2682,7 +2679,7 @@
         <v>125</v>
       </c>
       <c r="I59" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -2693,7 +2690,7 @@
         <v>175</v>
       </c>
       <c r="C60" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D60" t="s">
         <v>72</v>
@@ -2711,7 +2708,7 @@
         <v>125</v>
       </c>
       <c r="I60" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -2722,7 +2719,7 @@
         <v>176</v>
       </c>
       <c r="C61" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D61" t="s">
         <v>72</v>
@@ -2740,7 +2737,7 @@
         <v>125</v>
       </c>
       <c r="I61" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
@@ -2757,13 +2754,13 @@
         <v>74</v>
       </c>
       <c r="G62" t="s">
-        <v>178</v>
+        <v>72</v>
       </c>
       <c r="H62" t="s">
         <v>125</v>
       </c>
       <c r="I62" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
laga passing and receiving
</commit_message>
<xml_diff>
--- a/measurementInfo.xlsx
+++ b/measurementInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Notandi\Desktop\Measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA60187-614B-4CBC-AB5C-D746FE7D08B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3439E915-68C5-4241-AF53-302694177B1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CE7ABF46-5BCF-44D0-B551-448571CF2DF6}"/>
+    <workbookView xWindow="-21720" yWindow="2205" windowWidth="16410" windowHeight="11295" xr2:uid="{CE7ABF46-5BCF-44D0-B551-448571CF2DF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -68,9 +68,6 @@
     <t>Soccer Genius Game Action Running</t>
   </si>
   <si>
-    <t>Soccer Genius Passing and Reveiving</t>
-  </si>
-  <si>
     <t>Soccer Genius Dribbling</t>
   </si>
   <si>
@@ -612,6 +609,9 @@
   </si>
   <si>
     <t>soccer_passing_90deg_passing</t>
+  </si>
+  <si>
+    <t>Soccer Genius Passing and Receiving</t>
   </si>
 </sst>
 </file>
@@ -1026,1741 +1026,1741 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s">
         <v>70</v>
       </c>
-      <c r="C2" t="s">
-        <v>71</v>
-      </c>
       <c r="D2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F2" t="s">
         <v>73</v>
       </c>
-      <c r="F2" t="s">
-        <v>74</v>
-      </c>
       <c r="G2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>191</v>
       </c>
       <c r="B3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" t="s">
         <v>75</v>
       </c>
-      <c r="C3" t="s">
-        <v>76</v>
-      </c>
       <c r="D3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" t="s">
         <v>77</v>
       </c>
-      <c r="E3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F3" t="s">
-        <v>78</v>
-      </c>
       <c r="G3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B4" t="s">
         <v>185</v>
       </c>
-      <c r="B4" t="s">
-        <v>186</v>
-      </c>
       <c r="C4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" t="s">
         <v>77</v>
       </c>
-      <c r="E4" t="s">
-        <v>73</v>
-      </c>
-      <c r="F4" t="s">
-        <v>78</v>
-      </c>
       <c r="G4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" t="s">
         <v>80</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" t="s">
         <v>81</v>
       </c>
-      <c r="D5" t="s">
-        <v>77</v>
-      </c>
-      <c r="E5" t="s">
-        <v>73</v>
-      </c>
-      <c r="F5" t="s">
-        <v>82</v>
-      </c>
       <c r="G5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" t="s">
         <v>84</v>
       </c>
-      <c r="D7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E7" t="s">
-        <v>73</v>
-      </c>
-      <c r="F7" t="s">
-        <v>85</v>
-      </c>
       <c r="G7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" t="s">
+        <v>71</v>
+      </c>
+      <c r="E8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G8" t="s">
         <v>86</v>
       </c>
-      <c r="D8" t="s">
-        <v>72</v>
-      </c>
-      <c r="E8" t="s">
-        <v>73</v>
-      </c>
-      <c r="F8" t="s">
-        <v>85</v>
-      </c>
-      <c r="G8" t="s">
-        <v>87</v>
-      </c>
       <c r="H8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" t="s">
         <v>88</v>
       </c>
-      <c r="C9" t="s">
-        <v>89</v>
-      </c>
       <c r="D9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" t="s">
         <v>90</v>
       </c>
-      <c r="C10" t="s">
-        <v>91</v>
-      </c>
       <c r="D10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" t="s">
         <v>93</v>
       </c>
-      <c r="C11" t="s">
-        <v>94</v>
-      </c>
       <c r="D11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H11" t="s">
+        <v>177</v>
+      </c>
+      <c r="I11" t="s">
         <v>178</v>
-      </c>
-      <c r="I11" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I12" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C13" t="s">
         <v>96</v>
       </c>
-      <c r="C13" t="s">
-        <v>97</v>
-      </c>
       <c r="D13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" t="s">
         <v>98</v>
       </c>
-      <c r="C14" t="s">
-        <v>99</v>
-      </c>
       <c r="D14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E16" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" t="s">
         <v>73</v>
       </c>
-      <c r="F16" t="s">
-        <v>74</v>
-      </c>
       <c r="G16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" t="s">
         <v>77</v>
       </c>
-      <c r="E17" t="s">
-        <v>73</v>
-      </c>
-      <c r="F17" t="s">
-        <v>78</v>
-      </c>
       <c r="G17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H17" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I17" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" t="s">
+        <v>72</v>
+      </c>
+      <c r="F18" t="s">
         <v>77</v>
       </c>
-      <c r="E18" t="s">
-        <v>73</v>
-      </c>
-      <c r="F18" t="s">
-        <v>78</v>
-      </c>
       <c r="G18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H18" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I18" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" t="s">
+        <v>72</v>
+      </c>
+      <c r="F19" t="s">
         <v>77</v>
       </c>
-      <c r="E19" t="s">
-        <v>73</v>
-      </c>
-      <c r="F19" t="s">
-        <v>78</v>
-      </c>
       <c r="G19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H19" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I19" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" t="s">
         <v>104</v>
       </c>
-      <c r="C20" t="s">
-        <v>105</v>
-      </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H20" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I20" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C21" t="s">
         <v>106</v>
       </c>
-      <c r="C21" t="s">
-        <v>107</v>
-      </c>
       <c r="D21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G21" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I21" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" t="s">
         <v>108</v>
       </c>
-      <c r="C22" t="s">
-        <v>109</v>
-      </c>
       <c r="D22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G22" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H22" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I22" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B23" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" t="s">
         <v>110</v>
       </c>
-      <c r="C23" t="s">
-        <v>111</v>
-      </c>
       <c r="D23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G23" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H23" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I23" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B24" t="s">
+        <v>111</v>
+      </c>
+      <c r="C24" t="s">
         <v>112</v>
       </c>
-      <c r="C24" t="s">
-        <v>113</v>
-      </c>
       <c r="D24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H24" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I24" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C25" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D25" t="s">
+        <v>76</v>
+      </c>
+      <c r="E25" t="s">
+        <v>72</v>
+      </c>
+      <c r="F25" t="s">
         <v>77</v>
       </c>
-      <c r="E25" t="s">
-        <v>73</v>
-      </c>
-      <c r="F25" t="s">
-        <v>78</v>
-      </c>
       <c r="G25" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H25" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I25" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D26" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" t="s">
+        <v>72</v>
+      </c>
+      <c r="F26" t="s">
         <v>77</v>
       </c>
-      <c r="E26" t="s">
-        <v>73</v>
-      </c>
-      <c r="F26" t="s">
-        <v>78</v>
-      </c>
       <c r="G26" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H26" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I26" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F27" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G27" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H27" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I27" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H28" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I28" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B29" t="s">
+        <v>115</v>
+      </c>
+      <c r="C29" t="s">
         <v>116</v>
       </c>
-      <c r="C29" t="s">
-        <v>117</v>
-      </c>
       <c r="D29" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E29" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H29" t="s">
+        <v>177</v>
+      </c>
+      <c r="I29" t="s">
         <v>178</v>
-      </c>
-      <c r="I29" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B30" t="s">
+        <v>117</v>
+      </c>
+      <c r="C30" t="s">
         <v>118</v>
       </c>
-      <c r="C30" t="s">
-        <v>119</v>
-      </c>
       <c r="D30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G30" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H30" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I30" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B31" t="s">
+        <v>119</v>
+      </c>
+      <c r="C31" t="s">
         <v>120</v>
       </c>
-      <c r="C31" t="s">
-        <v>121</v>
-      </c>
       <c r="D31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E31" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H31" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I31" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D32" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F32" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G32" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H32" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I32" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C33" t="s">
+        <v>122</v>
+      </c>
+      <c r="D33" t="s">
+        <v>71</v>
+      </c>
+      <c r="E33" t="s">
         <v>123</v>
       </c>
-      <c r="D33" t="s">
-        <v>72</v>
-      </c>
-      <c r="E33" t="s">
-        <v>124</v>
-      </c>
       <c r="G33" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H33" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I33" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B34" t="s">
+        <v>125</v>
+      </c>
+      <c r="C34" t="s">
         <v>126</v>
       </c>
-      <c r="C34" t="s">
-        <v>127</v>
-      </c>
       <c r="D34" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E34" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F34" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G34" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B35" t="s">
+        <v>127</v>
+      </c>
+      <c r="C35" t="s">
         <v>128</v>
       </c>
-      <c r="C35" t="s">
-        <v>129</v>
-      </c>
       <c r="D35" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E35" t="s">
+        <v>72</v>
+      </c>
+      <c r="F35" t="s">
         <v>73</v>
       </c>
-      <c r="F35" t="s">
-        <v>74</v>
-      </c>
       <c r="G35" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H35" t="s">
+        <v>177</v>
+      </c>
+      <c r="I35" t="s">
         <v>178</v>
-      </c>
-      <c r="I35" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B36" t="s">
+        <v>129</v>
+      </c>
+      <c r="C36" t="s">
         <v>130</v>
       </c>
-      <c r="C36" t="s">
-        <v>131</v>
-      </c>
       <c r="D36" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E36" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F36" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G36" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H36" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I36" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B37" t="s">
+        <v>131</v>
+      </c>
+      <c r="C37" t="s">
         <v>132</v>
       </c>
-      <c r="C37" t="s">
-        <v>133</v>
-      </c>
       <c r="D37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E37" t="s">
+        <v>72</v>
+      </c>
+      <c r="F37" t="s">
         <v>73</v>
       </c>
-      <c r="F37" t="s">
-        <v>74</v>
-      </c>
       <c r="G37" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I37" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B38" t="s">
+        <v>133</v>
+      </c>
+      <c r="C38" t="s">
         <v>134</v>
       </c>
-      <c r="C38" t="s">
-        <v>135</v>
-      </c>
       <c r="D38" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F38" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G38" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H38" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I38" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B39" t="s">
+        <v>135</v>
+      </c>
+      <c r="C39" t="s">
         <v>136</v>
       </c>
-      <c r="C39" t="s">
-        <v>137</v>
-      </c>
       <c r="D39" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E39" t="s">
+        <v>72</v>
+      </c>
+      <c r="F39" t="s">
         <v>73</v>
       </c>
-      <c r="F39" t="s">
-        <v>74</v>
-      </c>
       <c r="G39" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H39" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I39" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B40" t="s">
+        <v>137</v>
+      </c>
+      <c r="C40" t="s">
         <v>138</v>
       </c>
-      <c r="C40" t="s">
-        <v>139</v>
-      </c>
       <c r="D40" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F40" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G40" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H40" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I40" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B41" t="s">
+        <v>139</v>
+      </c>
+      <c r="C41" t="s">
         <v>140</v>
       </c>
-      <c r="C41" t="s">
-        <v>141</v>
-      </c>
       <c r="D41" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E41" t="s">
+        <v>72</v>
+      </c>
+      <c r="F41" t="s">
         <v>73</v>
       </c>
-      <c r="F41" t="s">
-        <v>74</v>
-      </c>
       <c r="G41" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H41" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I41" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B42" t="s">
+        <v>141</v>
+      </c>
+      <c r="C42" t="s">
         <v>142</v>
       </c>
-      <c r="C42" t="s">
-        <v>143</v>
-      </c>
       <c r="D42" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E42" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F42" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I42" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B43" t="s">
+        <v>143</v>
+      </c>
+      <c r="C43" t="s">
         <v>144</v>
       </c>
-      <c r="C43" t="s">
-        <v>145</v>
-      </c>
       <c r="D43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E43" t="s">
+        <v>72</v>
+      </c>
+      <c r="F43" t="s">
         <v>73</v>
       </c>
-      <c r="F43" t="s">
-        <v>74</v>
-      </c>
       <c r="G43" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H43" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I43" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C44" t="s">
+        <v>145</v>
+      </c>
+      <c r="D44" t="s">
+        <v>71</v>
+      </c>
+      <c r="E44" t="s">
         <v>146</v>
       </c>
-      <c r="D44" t="s">
-        <v>72</v>
-      </c>
-      <c r="E44" t="s">
-        <v>147</v>
-      </c>
       <c r="G44" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H44" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I44" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B45" t="s">
+        <v>147</v>
+      </c>
+      <c r="C45" t="s">
         <v>148</v>
       </c>
-      <c r="C45" t="s">
-        <v>149</v>
-      </c>
       <c r="D45" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E45" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F45" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G45" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H45" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I45" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B46" t="s">
+        <v>149</v>
+      </c>
+      <c r="C46" t="s">
         <v>150</v>
       </c>
-      <c r="C46" t="s">
-        <v>151</v>
-      </c>
       <c r="D46" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E46" t="s">
+        <v>72</v>
+      </c>
+      <c r="F46" t="s">
         <v>73</v>
       </c>
-      <c r="F46" t="s">
-        <v>74</v>
-      </c>
       <c r="G46" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H46" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I46" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B47" t="s">
+        <v>151</v>
+      </c>
+      <c r="C47" t="s">
         <v>152</v>
       </c>
-      <c r="C47" t="s">
-        <v>153</v>
-      </c>
       <c r="D47" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E47" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F47" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G47" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I47" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B48" t="s">
+        <v>153</v>
+      </c>
+      <c r="C48" t="s">
         <v>154</v>
       </c>
-      <c r="C48" t="s">
-        <v>155</v>
-      </c>
       <c r="D48" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E48" t="s">
+        <v>72</v>
+      </c>
+      <c r="F48" t="s">
         <v>73</v>
       </c>
-      <c r="F48" t="s">
-        <v>74</v>
-      </c>
       <c r="G48" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H48" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I48" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B49" t="s">
+        <v>155</v>
+      </c>
+      <c r="C49" t="s">
         <v>156</v>
       </c>
-      <c r="C49" t="s">
-        <v>157</v>
-      </c>
       <c r="D49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E49" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F49" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G49" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H49" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I49" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B50" t="s">
+        <v>157</v>
+      </c>
+      <c r="C50" t="s">
         <v>158</v>
       </c>
-      <c r="C50" t="s">
-        <v>159</v>
-      </c>
       <c r="D50" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E50" t="s">
+        <v>72</v>
+      </c>
+      <c r="F50" t="s">
         <v>73</v>
       </c>
-      <c r="F50" t="s">
-        <v>74</v>
-      </c>
       <c r="G50" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H50" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I50" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B51" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C51" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D51" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E51" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F51" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G51" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I51" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B52" t="s">
+        <v>160</v>
+      </c>
+      <c r="C52" t="s">
         <v>161</v>
       </c>
-      <c r="C52" t="s">
-        <v>162</v>
-      </c>
       <c r="D52" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E52" t="s">
+        <v>72</v>
+      </c>
+      <c r="F52" t="s">
         <v>73</v>
       </c>
-      <c r="F52" t="s">
-        <v>74</v>
-      </c>
       <c r="G52" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H52" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I52" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B53" t="s">
+        <v>162</v>
+      </c>
+      <c r="C53" t="s">
         <v>163</v>
       </c>
-      <c r="C53" t="s">
-        <v>164</v>
-      </c>
       <c r="D53" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E53" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F53" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G53" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B54" t="s">
+        <v>164</v>
+      </c>
+      <c r="C54" t="s">
         <v>165</v>
       </c>
-      <c r="C54" t="s">
-        <v>166</v>
-      </c>
       <c r="D54" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E54" t="s">
+        <v>72</v>
+      </c>
+      <c r="F54" t="s">
         <v>73</v>
       </c>
-      <c r="F54" t="s">
-        <v>74</v>
-      </c>
       <c r="G54" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H54" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I54" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B55" t="s">
+        <v>166</v>
+      </c>
+      <c r="C55" t="s">
         <v>167</v>
       </c>
-      <c r="C55" t="s">
-        <v>168</v>
-      </c>
       <c r="D55" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E55" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F55" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G55" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H55" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I55" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B56" t="s">
+        <v>168</v>
+      </c>
+      <c r="C56" t="s">
         <v>169</v>
       </c>
-      <c r="C56" t="s">
-        <v>170</v>
-      </c>
       <c r="D56" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E56" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F56" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G56" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H56" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I56" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B57" t="s">
+        <v>170</v>
+      </c>
+      <c r="C57" t="s">
         <v>171</v>
       </c>
-      <c r="C57" t="s">
-        <v>172</v>
-      </c>
       <c r="D57" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E57" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F57" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G57" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H57" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I57" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B58" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C58" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D58" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E58" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F58" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G58" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H58" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I58" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B59" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C59" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D59" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E59" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F59" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G59" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H59" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I59" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B60" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C60" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D60" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E60" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F60" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G60" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H60" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I60" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B61" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C61" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D61" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E61" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F61" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G61" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H61" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I61" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C62" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E62" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F62" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G62" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H62" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I62" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
laga measurementInfo excelið (bæta við hvort myndir, description og myndbönd séu)
</commit_message>
<xml_diff>
--- a/measurementInfo.xlsx
+++ b/measurementInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Notandi\Desktop\Measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3439E915-68C5-4241-AF53-302694177B1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E69D397-AFA0-4930-A542-447A02D1D3DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="2205" windowWidth="16410" windowHeight="11295" xr2:uid="{CE7ABF46-5BCF-44D0-B551-448571CF2DF6}"/>
+    <workbookView xWindow="28680" yWindow="-4995" windowWidth="16440" windowHeight="28320" xr2:uid="{CE7ABF46-5BCF-44D0-B551-448571CF2DF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="195">
   <si>
     <t>title</t>
   </si>
@@ -612,6 +612,15 @@
   </si>
   <si>
     <t>Soccer Genius Passing and Receiving</t>
+  </si>
+  <si>
+    <t>image</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>video</t>
   </si>
 </sst>
 </file>
@@ -983,7 +992,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3204655E-E80D-446C-AF0B-3E0CCA1683CF}">
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40" bestFit="1" customWidth="1"/>
@@ -992,7 +1001,7 @@
     <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1020,8 +1029,17 @@
       <c r="I1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" t="s">
+        <v>193</v>
+      </c>
+      <c r="K1" t="s">
+        <v>192</v>
+      </c>
+      <c r="L1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1049,8 +1067,17 @@
       <c r="I2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>191</v>
       </c>
@@ -1078,8 +1105,17 @@
       <c r="I3" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>184</v>
       </c>
@@ -1107,8 +1143,17 @@
       <c r="I4" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1136,8 +1181,17 @@
       <c r="I5" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1159,8 +1213,17 @@
       <c r="I6" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1188,8 +1251,17 @@
       <c r="I7" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -1217,8 +1289,17 @@
       <c r="I8" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -1246,8 +1327,17 @@
       <c r="I9" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -1275,8 +1365,17 @@
       <c r="I10" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1304,8 +1403,17 @@
       <c r="I11" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1333,8 +1441,17 @@
       <c r="I12" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -1362,8 +1479,17 @@
       <c r="I13" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -1391,8 +1517,17 @@
       <c r="I14" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J14" t="b">
+        <v>1</v>
+      </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1420,8 +1555,17 @@
       <c r="I15" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J15" t="b">
+        <v>1</v>
+      </c>
+      <c r="K15" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -1449,8 +1593,17 @@
       <c r="I16" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -1478,8 +1631,17 @@
       <c r="I17" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -1507,8 +1669,17 @@
       <c r="I18" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J18" t="b">
+        <v>1</v>
+      </c>
+      <c r="K18" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -1536,8 +1707,17 @@
       <c r="I19" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -1565,8 +1745,17 @@
       <c r="I20" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -1594,8 +1783,17 @@
       <c r="I21" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J21" t="b">
+        <v>1</v>
+      </c>
+      <c r="K21" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -1623,8 +1821,17 @@
       <c r="I22" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J22" t="b">
+        <v>1</v>
+      </c>
+      <c r="K22" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -1652,8 +1859,17 @@
       <c r="I23" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J23" t="b">
+        <v>1</v>
+      </c>
+      <c r="K23" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -1681,8 +1897,17 @@
       <c r="I24" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J24" t="b">
+        <v>1</v>
+      </c>
+      <c r="K24" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -1710,8 +1935,17 @@
       <c r="I25" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J25" t="b">
+        <v>1</v>
+      </c>
+      <c r="K25" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -1739,8 +1973,17 @@
       <c r="I26" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J26" t="b">
+        <v>1</v>
+      </c>
+      <c r="K26" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>32</v>
       </c>
@@ -1768,8 +2011,17 @@
       <c r="I27" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J27" t="b">
+        <v>1</v>
+      </c>
+      <c r="K27" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>33</v>
       </c>
@@ -1797,8 +2049,17 @@
       <c r="I28" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J28" t="b">
+        <v>1</v>
+      </c>
+      <c r="K28" t="b">
+        <v>1</v>
+      </c>
+      <c r="L28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -1826,8 +2087,17 @@
       <c r="I29" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J29" t="b">
+        <v>1</v>
+      </c>
+      <c r="K29" t="b">
+        <v>1</v>
+      </c>
+      <c r="L29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -1855,8 +2125,17 @@
       <c r="I30" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J30" t="b">
+        <v>1</v>
+      </c>
+      <c r="K30" t="b">
+        <v>1</v>
+      </c>
+      <c r="L30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -1884,8 +2163,17 @@
       <c r="I31" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J31" t="b">
+        <v>1</v>
+      </c>
+      <c r="K31" t="b">
+        <v>1</v>
+      </c>
+      <c r="L31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -1913,8 +2201,17 @@
       <c r="I32" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J32" t="b">
+        <v>1</v>
+      </c>
+      <c r="K32" t="b">
+        <v>1</v>
+      </c>
+      <c r="L32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>38</v>
       </c>
@@ -1939,8 +2236,17 @@
       <c r="I33" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J33" t="b">
+        <v>1</v>
+      </c>
+      <c r="K33" t="b">
+        <v>1</v>
+      </c>
+      <c r="L33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>39</v>
       </c>
@@ -1968,8 +2274,17 @@
       <c r="I34" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J34" t="b">
+        <v>1</v>
+      </c>
+      <c r="K34" t="b">
+        <v>1</v>
+      </c>
+      <c r="L34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>40</v>
       </c>
@@ -1997,8 +2312,17 @@
       <c r="I35" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J35" t="b">
+        <v>1</v>
+      </c>
+      <c r="K35" t="b">
+        <v>1</v>
+      </c>
+      <c r="L35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>41</v>
       </c>
@@ -2026,8 +2350,17 @@
       <c r="I36" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J36" t="b">
+        <v>1</v>
+      </c>
+      <c r="K36" t="b">
+        <v>1</v>
+      </c>
+      <c r="L36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -2055,8 +2388,17 @@
       <c r="I37" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J37" t="b">
+        <v>1</v>
+      </c>
+      <c r="K37" t="b">
+        <v>1</v>
+      </c>
+      <c r="L37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -2084,8 +2426,17 @@
       <c r="I38" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J38" t="b">
+        <v>1</v>
+      </c>
+      <c r="K38" t="b">
+        <v>1</v>
+      </c>
+      <c r="L38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>44</v>
       </c>
@@ -2113,8 +2464,17 @@
       <c r="I39" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J39" t="b">
+        <v>1</v>
+      </c>
+      <c r="K39" t="b">
+        <v>1</v>
+      </c>
+      <c r="L39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>45</v>
       </c>
@@ -2142,8 +2502,17 @@
       <c r="I40" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J40" t="b">
+        <v>1</v>
+      </c>
+      <c r="K40" t="b">
+        <v>1</v>
+      </c>
+      <c r="L40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>46</v>
       </c>
@@ -2171,8 +2540,17 @@
       <c r="I41" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J41" t="b">
+        <v>1</v>
+      </c>
+      <c r="K41" t="b">
+        <v>1</v>
+      </c>
+      <c r="L41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>47</v>
       </c>
@@ -2200,8 +2578,17 @@
       <c r="I42" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J42" t="b">
+        <v>1</v>
+      </c>
+      <c r="K42" t="b">
+        <v>1</v>
+      </c>
+      <c r="L42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>48</v>
       </c>
@@ -2229,8 +2616,17 @@
       <c r="I43" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J43" t="b">
+        <v>1</v>
+      </c>
+      <c r="K43" t="b">
+        <v>1</v>
+      </c>
+      <c r="L43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -2252,8 +2648,17 @@
       <c r="I44" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J44" t="b">
+        <v>1</v>
+      </c>
+      <c r="K44" t="b">
+        <v>1</v>
+      </c>
+      <c r="L44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>50</v>
       </c>
@@ -2281,8 +2686,17 @@
       <c r="I45" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J45" t="b">
+        <v>1</v>
+      </c>
+      <c r="K45" t="b">
+        <v>1</v>
+      </c>
+      <c r="L45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>51</v>
       </c>
@@ -2310,8 +2724,17 @@
       <c r="I46" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J46" t="b">
+        <v>1</v>
+      </c>
+      <c r="K46" t="b">
+        <v>1</v>
+      </c>
+      <c r="L46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -2339,8 +2762,17 @@
       <c r="I47" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J47" t="b">
+        <v>1</v>
+      </c>
+      <c r="K47" t="b">
+        <v>1</v>
+      </c>
+      <c r="L47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>53</v>
       </c>
@@ -2368,8 +2800,17 @@
       <c r="I48" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J48" t="b">
+        <v>1</v>
+      </c>
+      <c r="K48" t="b">
+        <v>1</v>
+      </c>
+      <c r="L48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>54</v>
       </c>
@@ -2397,8 +2838,17 @@
       <c r="I49" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J49" t="b">
+        <v>1</v>
+      </c>
+      <c r="K49" t="b">
+        <v>1</v>
+      </c>
+      <c r="L49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>55</v>
       </c>
@@ -2426,8 +2876,17 @@
       <c r="I50" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J50" t="b">
+        <v>1</v>
+      </c>
+      <c r="K50" t="b">
+        <v>1</v>
+      </c>
+      <c r="L50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>56</v>
       </c>
@@ -2455,8 +2914,17 @@
       <c r="I51" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J51" t="b">
+        <v>1</v>
+      </c>
+      <c r="K51" t="b">
+        <v>1</v>
+      </c>
+      <c r="L51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -2484,8 +2952,17 @@
       <c r="I52" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J52" t="b">
+        <v>1</v>
+      </c>
+      <c r="K52" t="b">
+        <v>1</v>
+      </c>
+      <c r="L52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>58</v>
       </c>
@@ -2507,8 +2984,17 @@
       <c r="G53" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J53" t="b">
+        <v>1</v>
+      </c>
+      <c r="K53" t="b">
+        <v>1</v>
+      </c>
+      <c r="L53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>59</v>
       </c>
@@ -2536,8 +3022,17 @@
       <c r="I54" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J54" t="b">
+        <v>1</v>
+      </c>
+      <c r="K54" t="b">
+        <v>1</v>
+      </c>
+      <c r="L54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>60</v>
       </c>
@@ -2565,8 +3060,17 @@
       <c r="I55" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J55" t="b">
+        <v>1</v>
+      </c>
+      <c r="K55" t="b">
+        <v>1</v>
+      </c>
+      <c r="L55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>62</v>
       </c>
@@ -2594,8 +3098,17 @@
       <c r="I56" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J56" t="b">
+        <v>1</v>
+      </c>
+      <c r="K56" t="b">
+        <v>1</v>
+      </c>
+      <c r="L56" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>63</v>
       </c>
@@ -2623,8 +3136,17 @@
       <c r="I57" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J57" t="b">
+        <v>1</v>
+      </c>
+      <c r="K57" t="b">
+        <v>1</v>
+      </c>
+      <c r="L57" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>64</v>
       </c>
@@ -2652,8 +3174,17 @@
       <c r="I58" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J58" t="b">
+        <v>1</v>
+      </c>
+      <c r="K58" t="b">
+        <v>1</v>
+      </c>
+      <c r="L58" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>65</v>
       </c>
@@ -2681,8 +3212,17 @@
       <c r="I59" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J59" t="b">
+        <v>1</v>
+      </c>
+      <c r="K59" t="b">
+        <v>1</v>
+      </c>
+      <c r="L59" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>66</v>
       </c>
@@ -2710,8 +3250,17 @@
       <c r="I60" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J60" t="b">
+        <v>1</v>
+      </c>
+      <c r="K60" t="b">
+        <v>1</v>
+      </c>
+      <c r="L60" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>67</v>
       </c>
@@ -2739,8 +3288,17 @@
       <c r="I61" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J61" t="b">
+        <v>1</v>
+      </c>
+      <c r="K61" t="b">
+        <v>1</v>
+      </c>
+      <c r="L61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>68</v>
       </c>
@@ -2761,6 +3319,15 @@
       </c>
       <c r="I62" t="s">
         <v>180</v>
+      </c>
+      <c r="J62" t="b">
+        <v>0</v>
+      </c>
+      <c r="K62" t="b">
+        <v>0</v>
+      </c>
+      <c r="L62" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>